<commit_message>
feat: add optional column, PIX price built-in, dual subtotals (essential/optional/total)
</commit_message>
<xml_diff>
--- a/LISTA_DE_COMPRAS_ROVER.xlsx
+++ b/LISTA_DE_COMPRAS_ROVER.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
@@ -47,16 +53,23 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00B8860B"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="00375623"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -71,8 +84,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F9"/>
-        <bgColor rgb="00F2F5F9"/>
+        <fgColor rgb="00FFF9E6"/>
+        <bgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+        <bgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -122,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -139,16 +158,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -516,16 +560,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -551,15 +596,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Preço Unitário (R$)</t>
+          <t>Preço Unit. à vista (R$)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Subtotal (R$)</t>
+          <t>Subtotal à vista (R$)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Link Direto</t>
         </is>
@@ -583,13 +633,14 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>13.67</v>
+        <v>12.99</v>
       </c>
       <c r="F2" s="4">
         <f>D2*E2</f>
         <v/>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -613,13 +664,14 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>29.9</v>
+        <v>28.4</v>
       </c>
       <c r="F3" s="4">
         <f>D3*E3</f>
         <v/>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -643,13 +695,14 @@
         <v>4</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>39.9</v>
+        <v>37.9</v>
       </c>
       <c r="F4" s="4">
         <f>D4*E4</f>
         <v/>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -673,13 +726,14 @@
         <v>2</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
       <c r="F5" s="4">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -691,7 +745,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Módulo Driver Ponte H - L298N (Driver 1: Motores Esq.)</t>
+          <t>Módulo Driver Ponte H - L298N (Driver 1)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -703,13 +757,14 @@
         <v>1</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>14.9</v>
+        <v>14.15</v>
       </c>
       <c r="F6" s="4">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -721,7 +776,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Módulo Driver Ponte H - L298N (Driver 2: Motores Dir.)</t>
+          <t>Módulo Driver Ponte H - L298N (Driver 2)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -733,13 +788,14 @@
         <v>1</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>14.9</v>
+        <v>14.15</v>
       </c>
       <c r="F7" s="4">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -751,7 +807,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Conversor DC/DC Step Down Mini 560 5V (5A síncrono)</t>
+          <t>Conversor DC/DC Step Down Mini 560 5V (5A)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -763,13 +819,14 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>7.5</v>
+        <v>7.12</v>
       </c>
       <c r="F8" s="4">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -793,13 +850,14 @@
         <v>1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>66.41</v>
       </c>
       <c r="F9" s="4">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -823,73 +881,84 @@
         <v>1</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F10" s="4">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Módulo Buzzer 5V Passivo</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="F11" s="4">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="F11" s="9">
         <f>D11*E11</f>
         <v/>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Módulo WS2812 LED RGB (Barra 8 LEDs)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="F12" s="4">
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F12" s="9">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -913,13 +982,14 @@
         <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1.5</v>
+        <v>1.42</v>
       </c>
       <c r="F13" s="4">
         <f>D13*E13</f>
         <v/>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -943,13 +1013,14 @@
         <v>1</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>6.9</v>
+        <v>6.55</v>
       </c>
       <c r="F14" s="4">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -973,13 +1044,14 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F15" s="4">
         <f>D15*E15</f>
         <v/>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1003,13 +1075,14 @@
         <v>1</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>28.9</v>
+        <v>27.45</v>
       </c>
       <c r="F16" s="4">
         <f>D16*E16</f>
         <v/>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1039,7 +1112,8 @@
         <f>D17*E17</f>
         <v/>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1051,7 +1125,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Cartão MicroSD 32GB Sandisk Ultra A1 (FAT32 p/ ESP32)</t>
+          <t>Cartão MicroSD 32GB Sandisk Ultra A1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1069,126 +1143,129 @@
         <f>D18*E18</f>
         <v/>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Módulo Giroscópio MPU-6050 GY-521 (VR Head Tracking)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Módulo Giroscópio MPU-6050 GY-521 (VR)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="4" t="n">
+      <c r="D19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="9" t="n">
         <v>19.9</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="9">
         <f>D19*E19</f>
         <v/>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>Abrir Produto</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="21" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Subtotal RoboCore (Itens 1 a 15)</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="7">
-        <f>SUM(F2:F16)</f>
-        <v/>
-      </c>
-      <c r="G20" s="6" t="n"/>
-    </row>
-    <row r="21" ht="21" customHeight="1">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>RoboCore à vista no PIX (-5%)</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7">
-        <f>F20*0.95</f>
-        <v/>
-      </c>
-      <c r="G21" s="6" t="n"/>
-    </row>
-    <row r="22" ht="21" customHeight="1">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Subtotal Mercado Livre (Itens 16 a 18)</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="7">
-        <f>SUM(F17:F19)</f>
-        <v/>
-      </c>
-      <c r="G22" s="6" t="n"/>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Abrir Produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="14">
+        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F13+F14+F15+F16+F17+F18</f>
+        <v/>
+      </c>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="16">
+        <f>F11+F12+F19</f>
+        <v/>
+      </c>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="8" t="n"/>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL GERAL ESTIMADO (PIX RoboCore + ML)</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="9">
-        <f>F21+F22</f>
-        <v/>
-      </c>
-      <c r="G23" s="8" t="n"/>
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="18">
+        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19</f>
+        <v/>
+      </c>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1200,16 +1277,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1235,15 +1313,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Preço Unitário (R$)</t>
+          <t>Preço Unit. à vista (R$)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Subtotal (R$)</t>
+          <t>Subtotal à vista (R$)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Link Direto</t>
         </is>
@@ -1267,13 +1350,14 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>13.67</v>
+        <v>12.99</v>
       </c>
       <c r="F2" s="4">
         <f>D2*E2</f>
         <v/>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1297,13 +1381,14 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>49.9</v>
+        <v>47.4</v>
       </c>
       <c r="F3" s="4">
         <f>D3*E3</f>
         <v/>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1327,13 +1412,14 @@
         <v>1</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>6.9</v>
+        <v>6.55</v>
       </c>
       <c r="F4" s="4">
         <f>D4*E4</f>
         <v/>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1357,13 +1443,14 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>29.9</v>
+        <v>28.4</v>
       </c>
       <c r="F5" s="4">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1387,13 +1474,14 @@
         <v>4</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>39.9</v>
+        <v>37.9</v>
       </c>
       <c r="F6" s="4">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1417,13 +1505,14 @@
         <v>2</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
       <c r="F7" s="4">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1435,7 +1524,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Módulo Driver Ponte H - L298N (Driver 1: Esquerda)</t>
+          <t>Módulo Driver Ponte H - L298N (Driver 1)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1447,13 +1536,14 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>14.9</v>
+        <v>14.15</v>
       </c>
       <c r="F8" s="4">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1465,7 +1555,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Módulo Driver Ponte H - L298N (Driver 2: Direita)</t>
+          <t>Módulo Driver Ponte H - L298N (Driver 2)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1477,13 +1567,14 @@
         <v>1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>14.9</v>
+        <v>14.15</v>
       </c>
       <c r="F9" s="4">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1495,7 +1586,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Conversor DC/DC Step Down Mini 560 5V (5A síncrono)</t>
+          <t>Conversor DC/DC Step Down Mini 560 5V (5A)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1507,13 +1598,14 @@
         <v>1</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>7.5</v>
+        <v>7.12</v>
       </c>
       <c r="F10" s="4">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1537,13 +1629,14 @@
         <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>66.41</v>
       </c>
       <c r="F11" s="4">
         <f>D11*E11</f>
         <v/>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1567,73 +1660,84 @@
         <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="F12" s="4">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Módulo Buzzer 5V Passivo</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="F13" s="4">
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="F13" s="9">
         <f>D13*E13</f>
         <v/>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Módulo WS2812 LED RGB (Barra 8 LEDs)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="F14" s="4">
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F14" s="9">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1657,13 +1761,14 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1.5</v>
+        <v>1.42</v>
       </c>
       <c r="F15" s="4">
         <f>D15*E15</f>
         <v/>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1687,13 +1792,14 @@
         <v>1</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>6.9</v>
+        <v>6.55</v>
       </c>
       <c r="F16" s="4">
         <f>D16*E16</f>
         <v/>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1717,13 +1823,14 @@
         <v>1</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="F17" s="4">
         <f>D17*E17</f>
         <v/>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1747,13 +1854,14 @@
         <v>1</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>28.9</v>
+        <v>27.45</v>
       </c>
       <c r="F18" s="4">
         <f>D18*E18</f>
         <v/>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1783,7 +1891,8 @@
         <f>D19*E19</f>
         <v/>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1813,128 +1922,131 @@
         <f>D20*E20</f>
         <v/>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Módulo Giroscópio MPU-6050 GY-521 (VR Head Tracking)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Módulo Giroscópio MPU-6050 GY-521 (VR)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="4" t="n">
+      <c r="D21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9" t="n">
         <v>19.9</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="9">
         <f>D21*E21</f>
         <v/>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Abrir Produto</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="21" customHeight="1">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Subtotal RoboCore (Itens 1 a 17)</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="7">
-        <f>SUM(F2:F18)</f>
-        <v/>
-      </c>
-      <c r="G22" s="6" t="n"/>
-    </row>
-    <row r="23" ht="21" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>RoboCore à vista no PIX (-5%)</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="7">
-        <f>F22*0.95</f>
-        <v/>
-      </c>
-      <c r="G23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="21" customHeight="1">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Subtotal Mercado Livre (Itens 18 a 20)</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="7">
-        <f>SUM(F19:F21)</f>
-        <v/>
-      </c>
-      <c r="G24" s="6" t="n"/>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>Abrir Produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="8" customHeight="1">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="14">
+        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F15+F16+F17+F18+F19+F20</f>
+        <v/>
+      </c>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="16">
+        <f>F13+F14+F21</f>
+        <v/>
+      </c>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL GERAL ESTIMADO (PIX RoboCore + ML)</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="9">
-        <f>F23+F24</f>
-        <v/>
-      </c>
-      <c r="G25" s="8" t="n"/>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="18">
+        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19+F20+F21</f>
+        <v/>
+      </c>
+      <c r="G25" s="17" t="n"/>
+      <c r="H25" s="17" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: make prices and subtotals 100% dynamic via Excel formulas and 0/1 optional flags
</commit_message>
<xml_diff>
--- a/LISTA_DE_COMPRAS_ROVER.xlsx
+++ b/LISTA_DE_COMPRAS_ROVER.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,12 +40,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
@@ -53,14 +47,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B8860B"/>
-      <sz val="10"/>
+      <color rgb="00375623"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="11"/>
+      <color rgb="00B8860B"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -84,14 +78,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
-        <bgColor rgb="00FFF9E6"/>
+        <fgColor rgb="00E2F0D9"/>
+        <bgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
-        <bgColor rgb="00E2F0D9"/>
+        <fgColor rgb="00FFF9E6"/>
+        <bgColor rgb="00FFF9E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -141,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -158,47 +152,39 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF9E6"/>
+          <bgColor rgb="00FFF9E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -560,17 +546,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -596,20 +583,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Preço Unit. à vista (R$)</t>
+          <t>Preço Unitário (R$)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Subtotal à vista (R$)</t>
+          <t>Preço à Vista PIX (R$)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Opcional</t>
+          <t>Subtotal à Vista (R$)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional (0/1)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Link Direto</t>
         </is>
@@ -633,14 +625,20 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>12.99</v>
+        <v>13.67</v>
       </c>
       <c r="F2" s="4">
-        <f>D2*E2</f>
-        <v/>
-      </c>
-      <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr">
+        <f>IF(OR(C2="RoboCore", C2="Robo Core"), ROUND(E2*0.95, 2), E2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="4">
+        <f>D2*F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -664,14 +662,20 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>28.4</v>
+        <v>29.9</v>
       </c>
       <c r="F3" s="4">
-        <f>D3*E3</f>
-        <v/>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+        <f>IF(OR(C3="RoboCore", C3="Robo Core"), ROUND(E3*0.95, 2), E3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>D3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -695,14 +699,20 @@
         <v>4</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>37.9</v>
+        <v>39.9</v>
       </c>
       <c r="F4" s="4">
-        <f>D4*E4</f>
-        <v/>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+        <f>IF(OR(C4="RoboCore", C4="Robo Core"), ROUND(E4*0.95, 2), E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>D4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -726,14 +736,20 @@
         <v>2</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>9.4</v>
+        <v>9.9</v>
       </c>
       <c r="F5" s="4">
-        <f>D5*E5</f>
-        <v/>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+        <f>IF(OR(C5="RoboCore", C5="Robo Core"), ROUND(E5*0.95, 2), E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>D5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -757,14 +773,20 @@
         <v>1</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>14.15</v>
+        <v>14.9</v>
       </c>
       <c r="F6" s="4">
-        <f>D6*E6</f>
-        <v/>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+        <f>IF(OR(C6="RoboCore", C6="Robo Core"), ROUND(E6*0.95, 2), E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>D6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -788,14 +810,20 @@
         <v>1</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>14.15</v>
+        <v>14.9</v>
       </c>
       <c r="F7" s="4">
-        <f>D7*E7</f>
-        <v/>
-      </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+        <f>IF(OR(C7="RoboCore", C7="Robo Core"), ROUND(E7*0.95, 2), E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>D7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -819,14 +847,20 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>7.12</v>
+        <v>7.5</v>
       </c>
       <c r="F8" s="4">
-        <f>D8*E8</f>
-        <v/>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="6" t="inlineStr">
+        <f>IF(OR(C8="RoboCore", C8="Robo Core"), ROUND(E8*0.95, 2), E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>D8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -850,14 +884,20 @@
         <v>1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>66.41</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F9" s="4">
-        <f>D9*E9</f>
-        <v/>
-      </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr">
+        <f>IF(OR(C9="RoboCore", C9="Robo Core"), ROUND(E9*0.95, 2), E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>D9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -881,84 +921,94 @@
         <v>1</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="F10" s="4">
-        <f>D10*E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr">
+        <f>IF(OR(C10="RoboCore", C10="Robo Core"), ROUND(E10*0.95, 2), E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>D10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Módulo Buzzer 5V Passivo</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="F11" s="9">
-        <f>D11*E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F11" s="4">
+        <f>IF(OR(C11="RoboCore", C11="Robo Core"), ROUND(E11*0.95, 2), E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>D11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Módulo WS2812 LED RGB (Barra 8 LEDs)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="F12" s="9">
-        <f>D12*E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F12" s="4">
+        <f>IF(OR(C12="RoboCore", C12="Robo Core"), ROUND(E12*0.95, 2), E12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>D12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -982,14 +1032,20 @@
         <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1.42</v>
+        <v>1.5</v>
       </c>
       <c r="F13" s="4">
-        <f>D13*E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr">
+        <f>IF(OR(C13="RoboCore", C13="Robo Core"), ROUND(E13*0.95, 2), E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
+        <f>D13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1013,14 +1069,20 @@
         <v>1</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>6.55</v>
+        <v>6.9</v>
       </c>
       <c r="F14" s="4">
-        <f>D14*E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr">
+        <f>IF(OR(C14="RoboCore", C14="Robo Core"), ROUND(E14*0.95, 2), E14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>D14*F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1044,14 +1106,20 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>7.5</v>
+        <v>7.9</v>
       </c>
       <c r="F15" s="4">
-        <f>D15*E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr">
+        <f>IF(OR(C15="RoboCore", C15="Robo Core"), ROUND(E15*0.95, 2), E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>D15*F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1075,14 +1143,20 @@
         <v>1</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>27.45</v>
+        <v>28.9</v>
       </c>
       <c r="F16" s="4">
-        <f>D16*E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr">
+        <f>IF(OR(C16="RoboCore", C16="Robo Core"), ROUND(E16*0.95, 2), E16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>D16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1109,11 +1183,17 @@
         <v>119</v>
       </c>
       <c r="F17" s="4">
-        <f>D17*E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr">
+        <f>IF(OR(C17="RoboCore", C17="Robo Core"), ROUND(E17*0.95, 2), E17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="4">
+        <f>D17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1140,132 +1220,149 @@
         <v>49.9</v>
       </c>
       <c r="F18" s="4">
-        <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr">
+        <f>IF(OR(C18="RoboCore", C18="Robo Core"), ROUND(E18*0.95, 2), E18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="4">
+        <f>D18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Módulo Giroscópio MPU-6050 GY-521 (VR)</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="9" t="n">
+      <c r="D19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4" t="n">
         <v>19.9</v>
       </c>
-      <c r="F19" s="9">
-        <f>D19*E19</f>
-        <v/>
-      </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="F19" s="4">
+        <f>IF(OR(C19="RoboCore", C19="Robo Core"), ROUND(E19*0.95, 2), E19)</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
+        <f>D19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="20" ht="8" customHeight="1">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="14">
-        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F13+F14+F15+F16+F17+F18</f>
-        <v/>
-      </c>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="8">
+        <f>SUMIF(H$2:H$19, 0, G$2:G$19)</f>
+        <v/>
+      </c>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="15" t="n"/>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
         </is>
       </c>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="16">
-        <f>F11+F12+F19</f>
-        <v/>
-      </c>
-      <c r="G22" s="15" t="n"/>
-      <c r="H22" s="15" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="10">
+        <f>SUMIF(H$2:H$19, 1, G$2:G$19)</f>
+        <v/>
+      </c>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="17" t="n"/>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="18">
-        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19</f>
-        <v/>
-      </c>
-      <c r="G23" s="17" t="n"/>
-      <c r="H23" s="17" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="12">
+        <f>SUM(G$2:G$19)</f>
+        <v/>
+      </c>
+      <c r="H23" s="11" t="n"/>
+      <c r="I23" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:I19">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H2=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1277,17 +1374,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1313,20 +1411,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Preço Unit. à vista (R$)</t>
+          <t>Preço Unitário (R$)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Subtotal à vista (R$)</t>
+          <t>Preço à Vista PIX (R$)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Opcional</t>
+          <t>Subtotal à Vista (R$)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional (0/1)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Link Direto</t>
         </is>
@@ -1350,14 +1453,20 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>12.99</v>
+        <v>13.67</v>
       </c>
       <c r="F2" s="4">
-        <f>D2*E2</f>
-        <v/>
-      </c>
-      <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr">
+        <f>IF(OR(C2="RoboCore", C2="Robo Core"), ROUND(E2*0.95, 2), E2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="4">
+        <f>D2*F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1381,14 +1490,20 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>47.4</v>
+        <v>49.9</v>
       </c>
       <c r="F3" s="4">
-        <f>D3*E3</f>
-        <v/>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr">
+        <f>IF(OR(C3="RoboCore", C3="Robo Core"), ROUND(E3*0.95, 2), E3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>D3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1412,14 +1527,20 @@
         <v>1</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>6.55</v>
+        <v>6.9</v>
       </c>
       <c r="F4" s="4">
-        <f>D4*E4</f>
-        <v/>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr">
+        <f>IF(OR(C4="RoboCore", C4="Robo Core"), ROUND(E4*0.95, 2), E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>D4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1443,14 +1564,20 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>28.4</v>
+        <v>29.9</v>
       </c>
       <c r="F5" s="4">
-        <f>D5*E5</f>
-        <v/>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr">
+        <f>IF(OR(C5="RoboCore", C5="Robo Core"), ROUND(E5*0.95, 2), E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>D5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1474,14 +1601,20 @@
         <v>4</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>37.9</v>
+        <v>39.9</v>
       </c>
       <c r="F6" s="4">
-        <f>D6*E6</f>
-        <v/>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr">
+        <f>IF(OR(C6="RoboCore", C6="Robo Core"), ROUND(E6*0.95, 2), E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>D6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1505,14 +1638,20 @@
         <v>2</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>9.4</v>
+        <v>9.9</v>
       </c>
       <c r="F7" s="4">
-        <f>D7*E7</f>
-        <v/>
-      </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr">
+        <f>IF(OR(C7="RoboCore", C7="Robo Core"), ROUND(E7*0.95, 2), E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>D7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1536,14 +1675,20 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>14.15</v>
+        <v>14.9</v>
       </c>
       <c r="F8" s="4">
-        <f>D8*E8</f>
-        <v/>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="6" t="inlineStr">
+        <f>IF(OR(C8="RoboCore", C8="Robo Core"), ROUND(E8*0.95, 2), E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>D8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1567,14 +1712,20 @@
         <v>1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>14.15</v>
+        <v>14.9</v>
       </c>
       <c r="F9" s="4">
-        <f>D9*E9</f>
-        <v/>
-      </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr">
+        <f>IF(OR(C9="RoboCore", C9="Robo Core"), ROUND(E9*0.95, 2), E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>D9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1598,14 +1749,20 @@
         <v>1</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>7.12</v>
+        <v>7.5</v>
       </c>
       <c r="F10" s="4">
-        <f>D10*E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr">
+        <f>IF(OR(C10="RoboCore", C10="Robo Core"), ROUND(E10*0.95, 2), E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>D10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1629,14 +1786,20 @@
         <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>66.41</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F11" s="4">
-        <f>D11*E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr">
+        <f>IF(OR(C11="RoboCore", C11="Robo Core"), ROUND(E11*0.95, 2), E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>D11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1660,84 +1823,94 @@
         <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="F12" s="4">
-        <f>D12*E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr">
+        <f>IF(OR(C12="RoboCore", C12="Robo Core"), ROUND(E12*0.95, 2), E12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>D12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Módulo Buzzer 5V Passivo</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="F13" s="9">
-        <f>D13*E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F13" s="4">
+        <f>IF(OR(C13="RoboCore", C13="Robo Core"), ROUND(E13*0.95, 2), E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
+        <f>D13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Módulo WS2812 LED RGB (Barra 8 LEDs)</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>RoboCore</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="F14" s="9">
-        <f>D14*E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>RoboCore</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F14" s="4">
+        <f>IF(OR(C14="RoboCore", C14="Robo Core"), ROUND(E14*0.95, 2), E14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>D14*F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1761,14 +1934,20 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1.42</v>
+        <v>1.5</v>
       </c>
       <c r="F15" s="4">
-        <f>D15*E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr">
+        <f>IF(OR(C15="RoboCore", C15="Robo Core"), ROUND(E15*0.95, 2), E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>D15*F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1792,14 +1971,20 @@
         <v>1</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>6.55</v>
+        <v>6.9</v>
       </c>
       <c r="F16" s="4">
-        <f>D16*E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr">
+        <f>IF(OR(C16="RoboCore", C16="Robo Core"), ROUND(E16*0.95, 2), E16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>D16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1823,14 +2008,20 @@
         <v>1</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>7.5</v>
+        <v>7.9</v>
       </c>
       <c r="F17" s="4">
-        <f>D17*E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr">
+        <f>IF(OR(C17="RoboCore", C17="Robo Core"), ROUND(E17*0.95, 2), E17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="4">
+        <f>D17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1854,14 +2045,20 @@
         <v>1</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>27.45</v>
+        <v>28.9</v>
       </c>
       <c r="F18" s="4">
-        <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr">
+        <f>IF(OR(C18="RoboCore", C18="Robo Core"), ROUND(E18*0.95, 2), E18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="4">
+        <f>D18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1888,11 +2085,17 @@
         <v>389</v>
       </c>
       <c r="F19" s="4">
-        <f>D19*E19</f>
-        <v/>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr">
+        <f>IF(OR(C19="RoboCore", C19="Robo Core"), ROUND(E19*0.95, 2), E19)</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
+        <f>D19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
@@ -1919,134 +2122,151 @@
         <v>69.90000000000001</v>
       </c>
       <c r="F20" s="4">
-        <f>D20*E20</f>
-        <v/>
-      </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr">
+        <f>IF(OR(C20="RoboCore", C20="Robo Core"), ROUND(E20*0.95, 2), E20)</f>
+        <v/>
+      </c>
+      <c r="G20" s="4">
+        <f>D20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Módulo Giroscópio MPU-6050 GY-521 (VR)</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="9" t="n">
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4" t="n">
         <v>19.9</v>
       </c>
-      <c r="F21" s="9">
-        <f>D21*E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="F21" s="4">
+        <f>IF(OR(C21="RoboCore", C21="Robo Core"), ROUND(E21*0.95, 2), E21)</f>
+        <v/>
+      </c>
+      <c r="G21" s="4">
+        <f>D21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Abrir Produto</t>
         </is>
       </c>
     </row>
     <row r="22" ht="8" customHeight="1">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="12" t="n"/>
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="14">
-        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F15+F16+F17+F18+F19+F20</f>
-        <v/>
-      </c>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="8">
+        <f>SUMIF(H$2:H$21, 0, G$2:G$21)</f>
+        <v/>
+      </c>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="A24" s="9" t="n"/>
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
         </is>
       </c>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="16">
-        <f>F13+F14+F21</f>
-        <v/>
-      </c>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="10">
+        <f>SUMIF(H$2:H$21, 1, G$2:G$21)</f>
+        <v/>
+      </c>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="17" t="n"/>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="18">
-        <f>F2+F3+F4+F5+F6+F7+F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19+F20+F21</f>
-        <v/>
-      </c>
-      <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="12">
+        <f>SUM(G$2:G$21)</f>
+        <v/>
+      </c>
+      <c r="H25" s="11" t="n"/>
+      <c r="I25" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:I21">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H2=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
style: remove emojis and remove separate optional-only subtotal row
</commit_message>
<xml_diff>
--- a/LISTA_DE_COMPRAS_ROVER.xlsx
+++ b/LISTA_DE_COMPRAS_ROVER.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,17 +53,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B8860B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -80,12 +74,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2F0D9"/>
         <bgColor rgb="00E2F0D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
-        <bgColor rgb="00FFF9E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -159,16 +147,10 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -546,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1288,7 +1270,7 @@
       <c r="A21" s="7" t="n"/>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
+          <t>Total Essencial (sem opcionais) - à vista no PIX</t>
         </is>
       </c>
       <c r="C21" s="7" t="n"/>
@@ -1306,7 +1288,7 @@
       <c r="A22" s="9" t="n"/>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
+          <t>TOTAL GERAL (com opcionais) - à vista no PIX</t>
         </is>
       </c>
       <c r="C22" s="9" t="n"/>
@@ -1314,29 +1296,11 @@
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="9" t="n"/>
       <c r="G22" s="10">
-        <f>SUMIF(H$2:H$19, 1, G$2:G$19)</f>
+        <f>SUM(G$2:G$19)</f>
         <v/>
       </c>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="12">
-        <f>SUM(G$2:G$19)</f>
-        <v/>
-      </c>
-      <c r="H23" s="11" t="n"/>
-      <c r="I23" s="11" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I19">
@@ -1374,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2190,7 +2154,7 @@
       <c r="A23" s="7" t="n"/>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>✅  Total Essencial (sem opcionais) – à vista no PIX</t>
+          <t>Total Essencial (sem opcionais) - à vista no PIX</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>
@@ -2208,7 +2172,7 @@
       <c r="A24" s="9" t="n"/>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>⭐  Itens Opcionais (Buzzer, LEDs, Giroscópio)</t>
+          <t>TOTAL GERAL (com opcionais) - à vista no PIX</t>
         </is>
       </c>
       <c r="C24" s="9" t="n"/>
@@ -2216,29 +2180,11 @@
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
       <c r="G24" s="10">
-        <f>SUMIF(H$2:H$21, 1, G$2:G$21)</f>
+        <f>SUM(G$2:G$21)</f>
         <v/>
       </c>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>💰  TOTAL GERAL (com opcionais) – à vista no PIX</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="12">
-        <f>SUM(G$2:G$21)</f>
-        <v/>
-      </c>
-      <c r="H25" s="11" t="n"/>
-      <c r="I25" s="11" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I21">

</xml_diff>